<commit_message>
✨ Add warehouse management page and prepare for deployment
</commit_message>
<xml_diff>
--- a/uniform-assigner/debug_output.xlsx
+++ b/uniform-assigner/debug_output.xlsx
@@ -1613,7 +1613,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="193">
+  <cellXfs count="194">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2117,6 +2117,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="45" borderId="66" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="45" borderId="66" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2643,9 +2646,9 @@
           <t>郭婷心</t>
         </is>
       </c>
-      <c r="C3" s="168" t="inlineStr">
-        <is>
-          <t>F165/88-01</t>
+      <c r="C3" s="147" t="inlineStr">
+        <is>
+          <t>F165/88-02</t>
         </is>
       </c>
       <c r="D3" s="147" t="inlineStr">
@@ -2705,9 +2708,9 @@
           <t>江文欣</t>
         </is>
       </c>
-      <c r="C5" s="168" t="inlineStr">
-        <is>
-          <t>F165/88-02</t>
+      <c r="C5" s="147" t="inlineStr">
+        <is>
+          <t>F165/88-04</t>
         </is>
       </c>
       <c r="D5" s="147" t="inlineStr">
@@ -2838,9 +2841,9 @@
           <t>M175/88-02</t>
         </is>
       </c>
-      <c r="D9" s="168" t="inlineStr">
-        <is>
-          <t>M5702</t>
+      <c r="D9" s="147" t="inlineStr">
+        <is>
+          <t>M5701</t>
         </is>
       </c>
       <c r="E9" s="147" t="inlineStr">
@@ -2908,9 +2911,9 @@
           <t>M180/92-03</t>
         </is>
       </c>
-      <c r="D11" s="168" t="inlineStr">
-        <is>
-          <t>M5703</t>
+      <c r="D11" s="147" t="inlineStr">
+        <is>
+          <t>M5704</t>
         </is>
       </c>
       <c r="E11" s="147" t="inlineStr">
@@ -3039,9 +3042,9 @@
           <t>顾铭文</t>
         </is>
       </c>
-      <c r="C15" s="168" t="inlineStr">
-        <is>
-          <t>M185/100-01</t>
+      <c r="C15" s="147" t="inlineStr">
+        <is>
+          <t>M185/100-02</t>
         </is>
       </c>
       <c r="D15" s="147" t="inlineStr">
@@ -3206,9 +3209,9 @@
           <t>吕凯进</t>
         </is>
       </c>
-      <c r="C20" s="154" t="inlineStr">
-        <is>
-          <t>M175/92-02</t>
+      <c r="C20" s="168" t="inlineStr">
+        <is>
+          <t>M175/92-01</t>
         </is>
       </c>
       <c r="D20" s="154" t="inlineStr">
@@ -3226,9 +3229,9 @@
           <t>M20</t>
         </is>
       </c>
-      <c r="G20" s="155" t="inlineStr">
-        <is>
-          <t>和戴傲共用礼帽</t>
+      <c r="G20" s="169" t="inlineStr">
+        <is>
+          <t>和潘睿、楼震霆共用礼服</t>
         </is>
       </c>
     </row>
@@ -3276,9 +3279,9 @@
           <t>柳洋</t>
         </is>
       </c>
-      <c r="C22" s="168" t="inlineStr">
-        <is>
-          <t>M180/96-07</t>
+      <c r="C22" s="154" t="inlineStr">
+        <is>
+          <t>M180/96-02</t>
         </is>
       </c>
       <c r="D22" s="154" t="inlineStr">
@@ -3346,9 +3349,9 @@
           <t>王梓丞</t>
         </is>
       </c>
-      <c r="C24" s="168" t="inlineStr">
-        <is>
-          <t>M180/96-07</t>
+      <c r="C24" s="154" t="inlineStr">
+        <is>
+          <t>M180/96-04</t>
         </is>
       </c>
       <c r="D24" s="154" t="inlineStr">
@@ -3418,7 +3421,7 @@
       </c>
       <c r="C26" s="168" t="inlineStr">
         <is>
-          <t>M180/96-05</t>
+          <t>M180/96-07</t>
         </is>
       </c>
       <c r="D26" s="154" t="inlineStr">
@@ -3436,9 +3439,9 @@
           <t>M21</t>
         </is>
       </c>
-      <c r="G26" s="154" t="inlineStr">
-        <is>
-          <t>和钱俊宇、努尔加娜特共用礼服</t>
+      <c r="G26" s="168" t="inlineStr">
+        <is>
+          <t>和孜英、张煜琦共用礼服</t>
         </is>
       </c>
     </row>
@@ -3622,9 +3625,9 @@
           <t>祁子谦</t>
         </is>
       </c>
-      <c r="C32" s="168" t="inlineStr">
-        <is>
-          <t>F170/84-01</t>
+      <c r="C32" s="159" t="inlineStr">
+        <is>
+          <t>F170/84-03</t>
         </is>
       </c>
       <c r="D32" s="159" t="inlineStr">
@@ -3767,9 +3770,9 @@
           <t>M180/96-01</t>
         </is>
       </c>
-      <c r="D36" s="168" t="inlineStr">
-        <is>
-          <t>M5804</t>
+      <c r="D36" s="159" t="inlineStr">
+        <is>
+          <t>M5805</t>
         </is>
       </c>
       <c r="E36" s="159" t="inlineStr">
@@ -3968,9 +3971,9 @@
           <t>王雨梦</t>
         </is>
       </c>
-      <c r="C42" s="168" t="inlineStr">
-        <is>
-          <t>F165/88-04</t>
+      <c r="C42" s="162" t="inlineStr">
+        <is>
+          <t>F165/88-01</t>
         </is>
       </c>
       <c r="D42" s="162" t="inlineStr">
@@ -4069,9 +4072,9 @@
           <t>俞恩祺</t>
         </is>
       </c>
-      <c r="C45" s="168" t="inlineStr">
-        <is>
-          <t>F175/92-02</t>
+      <c r="C45" s="162" t="inlineStr">
+        <is>
+          <t>F175/92-01</t>
         </is>
       </c>
       <c r="D45" s="162" t="inlineStr">
@@ -4486,9 +4489,9 @@
           <t>F170/92-02</t>
         </is>
       </c>
-      <c r="D57" s="168" t="inlineStr">
-        <is>
-          <t>F5602</t>
+      <c r="D57" s="166" t="inlineStr">
+        <is>
+          <t>F5601</t>
         </is>
       </c>
       <c r="E57" s="166" t="inlineStr">
@@ -4521,9 +4524,9 @@
           <t>M175/88-01</t>
         </is>
       </c>
-      <c r="D58" s="166" t="inlineStr">
-        <is>
-          <t>M5601</t>
+      <c r="D58" s="168" t="inlineStr">
+        <is>
+          <t>M5701</t>
         </is>
       </c>
       <c r="E58" s="166" t="inlineStr">
@@ -4536,9 +4539,9 @@
           <t>M01</t>
         </is>
       </c>
-      <c r="G58" s="167" t="inlineStr">
-        <is>
-          <t>和叶栩浩共用礼帽</t>
+      <c r="G58" s="169" t="inlineStr">
+        <is>
+          <t>和吴昕桐、韦景浩、文科共用礼帽</t>
         </is>
       </c>
     </row>
@@ -4622,9 +4625,9 @@
           <t>M175/96-03</t>
         </is>
       </c>
-      <c r="D61" s="168" t="inlineStr">
-        <is>
-          <t>M5703</t>
+      <c r="D61" s="166" t="inlineStr">
+        <is>
+          <t>M5701</t>
         </is>
       </c>
       <c r="E61" s="166" t="inlineStr">
@@ -4762,9 +4765,9 @@
           <t>M185/100-02</t>
         </is>
       </c>
-      <c r="D65" s="168" t="inlineStr">
-        <is>
-          <t>M5902</t>
+      <c r="D65" s="166" t="inlineStr">
+        <is>
+          <t>M5903</t>
         </is>
       </c>
       <c r="E65" s="166" t="inlineStr">
@@ -4834,28 +4837,28 @@
           <t>礼服腰带摆放</t>
         </is>
       </c>
-      <c r="B1" s="169" t="n"/>
-      <c r="C1" s="169" t="n"/>
-      <c r="D1" s="169" t="n"/>
-      <c r="E1" s="169" t="n"/>
-      <c r="F1" s="169" t="n"/>
-      <c r="G1" s="169" t="n"/>
-      <c r="H1" s="169" t="n"/>
-      <c r="I1" s="169" t="n"/>
-      <c r="J1" s="169" t="n"/>
-      <c r="K1" s="169" t="n"/>
-      <c r="L1" s="169" t="n"/>
-      <c r="M1" s="169" t="n"/>
-      <c r="N1" s="169" t="n"/>
-      <c r="O1" s="169" t="n"/>
-      <c r="P1" s="169" t="n"/>
-      <c r="Q1" s="169" t="n"/>
-      <c r="R1" s="169" t="n"/>
-      <c r="S1" s="169" t="n"/>
-      <c r="T1" s="169" t="n"/>
-      <c r="U1" s="169" t="n"/>
-      <c r="V1" s="169" t="n"/>
-      <c r="W1" s="169" t="n"/>
+      <c r="B1" s="170" t="n"/>
+      <c r="C1" s="170" t="n"/>
+      <c r="D1" s="170" t="n"/>
+      <c r="E1" s="170" t="n"/>
+      <c r="F1" s="170" t="n"/>
+      <c r="G1" s="170" t="n"/>
+      <c r="H1" s="170" t="n"/>
+      <c r="I1" s="170" t="n"/>
+      <c r="J1" s="170" t="n"/>
+      <c r="K1" s="170" t="n"/>
+      <c r="L1" s="170" t="n"/>
+      <c r="M1" s="170" t="n"/>
+      <c r="N1" s="170" t="n"/>
+      <c r="O1" s="170" t="n"/>
+      <c r="P1" s="170" t="n"/>
+      <c r="Q1" s="170" t="n"/>
+      <c r="R1" s="170" t="n"/>
+      <c r="S1" s="170" t="n"/>
+      <c r="T1" s="170" t="n"/>
+      <c r="U1" s="170" t="n"/>
+      <c r="V1" s="170" t="n"/>
+      <c r="W1" s="170" t="n"/>
       <c r="X1" s="56" t="n"/>
       <c r="Y1" s="96" t="inlineStr">
         <is>
@@ -4983,7 +4986,7 @@
           <t>李泽一</t>
         </is>
       </c>
-      <c r="E3" s="170" t="inlineStr">
+      <c r="E3" s="171" t="inlineStr">
         <is>
           <t>二</t>
         </is>
@@ -5003,7 +5006,7 @@
           <t>李诗诗、王雨梦</t>
         </is>
       </c>
-      <c r="I3" s="170" t="inlineStr">
+      <c r="I3" s="171" t="inlineStr">
         <is>
           <t>三</t>
         </is>
@@ -5035,7 +5038,7 @@
           <t>方嫄</t>
         </is>
       </c>
-      <c r="Q3" s="170" t="inlineStr">
+      <c r="Q3" s="171" t="inlineStr">
         <is>
           <t>五</t>
         </is>
@@ -5055,7 +5058,7 @@
           <t>艾克达、卢格妤</t>
         </is>
       </c>
-      <c r="U3" s="171" t="inlineStr">
+      <c r="U3" s="172" t="inlineStr">
         <is>
           <t>六</t>
         </is>
@@ -5070,7 +5073,7 @@
       <c r="Y3" s="11" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="172" t="n"/>
+      <c r="A4" s="173" t="n"/>
       <c r="B4" s="111" t="inlineStr">
         <is>
           <t>F165/80-02</t>
@@ -5081,7 +5084,7 @@
           <t>F02</t>
         </is>
       </c>
-      <c r="E4" s="172" t="n"/>
+      <c r="E4" s="173" t="n"/>
       <c r="F4" s="111" t="inlineStr">
         <is>
           <t>F165/88-02</t>
@@ -5097,7 +5100,7 @@
           <t>郭婷心</t>
         </is>
       </c>
-      <c r="I4" s="172" t="n"/>
+      <c r="I4" s="173" t="n"/>
       <c r="J4" s="111" t="inlineStr">
         <is>
           <t>F175/92-01</t>
@@ -5113,7 +5116,7 @@
           <t>俞恩祺、陈涵予</t>
         </is>
       </c>
-      <c r="M4" s="173" t="n"/>
+      <c r="M4" s="174" t="n"/>
       <c r="N4" s="111" t="inlineStr">
         <is>
           <t>F170/84-02</t>
@@ -5129,7 +5132,7 @@
           <t>柯天翊</t>
         </is>
       </c>
-      <c r="Q4" s="172" t="n"/>
+      <c r="Q4" s="173" t="n"/>
       <c r="R4" s="111" t="inlineStr">
         <is>
           <t>F170/92-02</t>
@@ -5155,7 +5158,7 @@
       <c r="Y4" s="11" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="172" t="n"/>
+      <c r="A5" s="173" t="n"/>
       <c r="B5" s="111" t="inlineStr">
         <is>
           <t>F165/84-01</t>
@@ -5171,7 +5174,7 @@
           <t>林珩</t>
         </is>
       </c>
-      <c r="E5" s="172" t="n"/>
+      <c r="E5" s="173" t="n"/>
       <c r="F5" s="111" t="inlineStr">
         <is>
           <t>F165/88-03</t>
@@ -5187,7 +5190,7 @@
           <t>岳佳凝、吴桐</t>
         </is>
       </c>
-      <c r="I5" s="172" t="n"/>
+      <c r="I5" s="173" t="n"/>
       <c r="J5" s="117" t="inlineStr">
         <is>
           <t>F175/92-02</t>
@@ -5195,7 +5198,7 @@
       </c>
       <c r="K5" s="112" t="n"/>
       <c r="L5" s="11" t="n"/>
-      <c r="M5" s="173" t="n"/>
+      <c r="M5" s="174" t="n"/>
       <c r="N5" s="111" t="inlineStr">
         <is>
           <t>F170/84-03</t>
@@ -5211,7 +5214,7 @@
           <t>祁子谦、段茗萱</t>
         </is>
       </c>
-      <c r="Q5" s="172" t="n"/>
+      <c r="Q5" s="173" t="n"/>
       <c r="R5" s="111" t="inlineStr">
         <is>
           <t>M180/96-01</t>
@@ -5237,7 +5240,7 @@
       <c r="Y5" s="11" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="172" t="n"/>
+      <c r="A6" s="173" t="n"/>
       <c r="B6" s="111" t="inlineStr">
         <is>
           <t>F165/84-02</t>
@@ -5253,7 +5256,7 @@
           <t>方佳瑶</t>
         </is>
       </c>
-      <c r="E6" s="172" t="n"/>
+      <c r="E6" s="173" t="n"/>
       <c r="F6" s="111" t="inlineStr">
         <is>
           <t>F165/88-04</t>
@@ -5269,7 +5272,7 @@
           <t>江文欣、董欢瑶</t>
         </is>
       </c>
-      <c r="I6" s="172" t="n"/>
+      <c r="I6" s="173" t="n"/>
       <c r="J6" s="111" t="inlineStr">
         <is>
           <t>M175/96-01</t>
@@ -5285,7 +5288,7 @@
           <t>张鹏</t>
         </is>
       </c>
-      <c r="M6" s="173" t="n"/>
+      <c r="M6" s="174" t="n"/>
       <c r="N6" s="111" t="inlineStr">
         <is>
           <t>F170/84-04</t>
@@ -5301,7 +5304,7 @@
           <t>张艺</t>
         </is>
       </c>
-      <c r="Q6" s="172" t="n"/>
+      <c r="Q6" s="173" t="n"/>
       <c r="R6" s="111" t="inlineStr">
         <is>
           <t>M180/96-02</t>
@@ -5327,7 +5330,7 @@
       <c r="Y6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="172" t="n"/>
+      <c r="A7" s="173" t="n"/>
       <c r="B7" s="111" t="inlineStr">
         <is>
           <t>F165/84-03</t>
@@ -5343,7 +5346,7 @@
           <t>纪博雅</t>
         </is>
       </c>
-      <c r="E7" s="172" t="n"/>
+      <c r="E7" s="173" t="n"/>
       <c r="F7" s="111" t="inlineStr">
         <is>
           <t>F175/88-01</t>
@@ -5359,7 +5362,7 @@
           <t>马欣雅</t>
         </is>
       </c>
-      <c r="I7" s="172" t="n"/>
+      <c r="I7" s="173" t="n"/>
       <c r="J7" s="111" t="inlineStr">
         <is>
           <t>M175/96-02</t>
@@ -5375,7 +5378,7 @@
           <t>叶宇轩</t>
         </is>
       </c>
-      <c r="M7" s="173" t="n"/>
+      <c r="M7" s="174" t="n"/>
       <c r="N7" s="115" t="inlineStr">
         <is>
           <t>F170/84-05</t>
@@ -5383,7 +5386,7 @@
       </c>
       <c r="O7" s="112" t="n"/>
       <c r="P7" s="46" t="n"/>
-      <c r="Q7" s="172" t="n"/>
+      <c r="Q7" s="173" t="n"/>
       <c r="R7" s="120" t="inlineStr">
         <is>
           <t>M180/96-03</t>
@@ -5409,7 +5412,7 @@
       <c r="Y7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="172" t="n"/>
+      <c r="A8" s="173" t="n"/>
       <c r="B8" s="117" t="inlineStr">
         <is>
           <t>F165/84-04</t>
@@ -5417,7 +5420,7 @@
       </c>
       <c r="C8" s="121" t="n"/>
       <c r="D8" s="65" t="n"/>
-      <c r="E8" s="172" t="n"/>
+      <c r="E8" s="173" t="n"/>
       <c r="F8" s="111" t="inlineStr">
         <is>
           <t>M180/92-05</t>
@@ -5433,7 +5436,7 @@
           <t>李思齐</t>
         </is>
       </c>
-      <c r="I8" s="172" t="n"/>
+      <c r="I8" s="173" t="n"/>
       <c r="J8" s="111" t="inlineStr">
         <is>
           <t>M175/96-03</t>
@@ -5449,7 +5452,7 @@
           <t>文科</t>
         </is>
       </c>
-      <c r="M8" s="173" t="n"/>
+      <c r="M8" s="174" t="n"/>
       <c r="N8" s="111" t="inlineStr">
         <is>
           <t>F170/84-06</t>
@@ -5465,7 +5468,7 @@
           <t>韩雅丽</t>
         </is>
       </c>
-      <c r="Q8" s="172" t="n"/>
+      <c r="Q8" s="173" t="n"/>
       <c r="R8" s="111" t="inlineStr">
         <is>
           <t>M180/96-04</t>
@@ -5491,7 +5494,7 @@
       <c r="Y8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="172" t="n"/>
+      <c r="A9" s="173" t="n"/>
       <c r="B9" s="115" t="inlineStr">
         <is>
           <t>F165/84-05</t>
@@ -5499,7 +5502,7 @@
       </c>
       <c r="C9" s="112" t="n"/>
       <c r="D9" s="65" t="n"/>
-      <c r="E9" s="172" t="n"/>
+      <c r="E9" s="173" t="n"/>
       <c r="F9" s="111" t="inlineStr">
         <is>
           <t>M180/92-06</t>
@@ -5515,7 +5518,7 @@
           <t>叶栩浩</t>
         </is>
       </c>
-      <c r="I9" s="172" t="n"/>
+      <c r="I9" s="173" t="n"/>
       <c r="J9" s="120" t="inlineStr">
         <is>
           <t>M175/96-04</t>
@@ -5531,7 +5534,7 @@
           <t>冯敬栩</t>
         </is>
       </c>
-      <c r="M9" s="173" t="n"/>
+      <c r="M9" s="174" t="n"/>
       <c r="N9" s="111" t="inlineStr">
         <is>
           <t>F170/88-01</t>
@@ -5547,7 +5550,7 @@
           <t>施东隅</t>
         </is>
       </c>
-      <c r="Q9" s="172" t="n"/>
+      <c r="Q9" s="173" t="n"/>
       <c r="R9" s="111" t="inlineStr">
         <is>
           <t>M180/96-05</t>
@@ -5581,7 +5584,7 @@
       <c r="Y9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="172" t="n"/>
+      <c r="A10" s="173" t="n"/>
       <c r="B10" s="111" t="inlineStr">
         <is>
           <t>M175/88-01</t>
@@ -5597,7 +5600,7 @@
           <t>陈思骆</t>
         </is>
       </c>
-      <c r="E10" s="172" t="n"/>
+      <c r="E10" s="173" t="n"/>
       <c r="F10" s="111" t="inlineStr">
         <is>
           <t>M180/92-07</t>
@@ -5605,7 +5608,7 @@
       </c>
       <c r="G10" s="124" t="n"/>
       <c r="H10" s="125" t="n"/>
-      <c r="I10" s="172" t="n"/>
+      <c r="I10" s="173" t="n"/>
       <c r="J10" s="111" t="inlineStr">
         <is>
           <t>M180/92-01</t>
@@ -5621,7 +5624,7 @@
           <t>张嘉靖</t>
         </is>
       </c>
-      <c r="M10" s="173" t="n"/>
+      <c r="M10" s="174" t="n"/>
       <c r="N10" s="111" t="inlineStr">
         <is>
           <t>F170/88-02</t>
@@ -5637,7 +5640,7 @@
           <t>呼岳洋、章芮容</t>
         </is>
       </c>
-      <c r="Q10" s="172" t="n"/>
+      <c r="Q10" s="173" t="n"/>
       <c r="R10" s="111" t="inlineStr">
         <is>
           <t>M180/100-01</t>
@@ -5671,7 +5674,7 @@
       <c r="Y10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="172" t="n"/>
+      <c r="A11" s="173" t="n"/>
       <c r="B11" s="120" t="inlineStr">
         <is>
           <t>M175/88-02</t>
@@ -5687,7 +5690,7 @@
           <t>吴昕桐</t>
         </is>
       </c>
-      <c r="E11" s="172" t="n"/>
+      <c r="E11" s="173" t="n"/>
       <c r="F11" s="111" t="inlineStr">
         <is>
           <t>M180/92-08</t>
@@ -5695,7 +5698,7 @@
       </c>
       <c r="G11" s="112" t="n"/>
       <c r="H11" s="116" t="n"/>
-      <c r="I11" s="172" t="n"/>
+      <c r="I11" s="173" t="n"/>
       <c r="J11" s="111" t="inlineStr">
         <is>
           <t>M180/92-02</t>
@@ -5711,7 +5714,7 @@
           <t>肖玉茂</t>
         </is>
       </c>
-      <c r="M11" s="173" t="n"/>
+      <c r="M11" s="174" t="n"/>
       <c r="N11" s="117" t="inlineStr">
         <is>
           <t>F170/88-03</t>
@@ -5719,7 +5722,7 @@
       </c>
       <c r="O11" s="112" t="n"/>
       <c r="P11" s="108" t="n"/>
-      <c r="Q11" s="172" t="n"/>
+      <c r="Q11" s="173" t="n"/>
       <c r="R11" s="111" t="inlineStr">
         <is>
           <t>M180/92-09</t>
@@ -5745,7 +5748,7 @@
       <c r="Y11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="172" t="n"/>
+      <c r="A12" s="173" t="n"/>
       <c r="B12" s="111" t="inlineStr">
         <is>
           <t>M175/92-01</t>
@@ -5761,7 +5764,7 @@
           <t>楼震霆、潘睿</t>
         </is>
       </c>
-      <c r="E12" s="172" t="n"/>
+      <c r="E12" s="173" t="n"/>
       <c r="F12" s="117" t="inlineStr">
         <is>
           <t>M180/92-10</t>
@@ -5769,7 +5772,7 @@
       </c>
       <c r="G12" s="112" t="n"/>
       <c r="H12" s="11" t="n"/>
-      <c r="I12" s="172" t="n"/>
+      <c r="I12" s="173" t="n"/>
       <c r="J12" s="111" t="inlineStr">
         <is>
           <t>M180/92-03</t>
@@ -5785,7 +5788,7 @@
           <t>夏瑞泽</t>
         </is>
       </c>
-      <c r="M12" s="173" t="n"/>
+      <c r="M12" s="174" t="n"/>
       <c r="N12" s="111" t="inlineStr">
         <is>
           <t>M180/96-06</t>
@@ -5801,7 +5804,7 @@
           <t>钱俊宇、努尔加娜特、张子恒</t>
         </is>
       </c>
-      <c r="Q12" s="172" t="n"/>
+      <c r="Q12" s="173" t="n"/>
       <c r="R12" s="126" t="inlineStr">
         <is>
           <t>M180/92-12</t>
@@ -5827,7 +5830,7 @@
       <c r="Y12" s="11" t="n"/>
     </row>
     <row r="13" ht="14.75" customHeight="1" s="113">
-      <c r="A13" s="174" t="n"/>
+      <c r="A13" s="175" t="n"/>
       <c r="B13" s="128" t="inlineStr">
         <is>
           <t>M175/92-02</t>
@@ -5843,7 +5846,7 @@
           <t>吕凯进</t>
         </is>
       </c>
-      <c r="E13" s="175" t="n"/>
+      <c r="E13" s="176" t="n"/>
       <c r="F13" s="131" t="inlineStr">
         <is>
           <t>M180/92-11</t>
@@ -5851,7 +5854,7 @@
       </c>
       <c r="G13" s="132" t="n"/>
       <c r="H13" s="133" t="n"/>
-      <c r="I13" s="175" t="n"/>
+      <c r="I13" s="176" t="n"/>
       <c r="J13" s="128" t="inlineStr">
         <is>
           <t>M180/92-04</t>
@@ -5867,7 +5870,7 @@
           <t>胡思源</t>
         </is>
       </c>
-      <c r="M13" s="176" t="n"/>
+      <c r="M13" s="177" t="n"/>
       <c r="N13" s="128" t="inlineStr">
         <is>
           <t>M180/96-07</t>
@@ -5883,11 +5886,11 @@
           <t>张煜琦、孜英</t>
         </is>
       </c>
-      <c r="Q13" s="175" t="n"/>
+      <c r="Q13" s="176" t="n"/>
       <c r="R13" s="136" t="n"/>
       <c r="S13" s="137" t="n"/>
       <c r="T13" s="138" t="n"/>
-      <c r="U13" s="177" t="n"/>
+      <c r="U13" s="178" t="n"/>
       <c r="V13" s="139" t="inlineStr">
         <is>
           <t>M185/100-03</t>
@@ -5928,22 +5931,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A1" s="178" t="inlineStr">
+      <c r="A1" s="179" t="inlineStr">
         <is>
           <t>礼帽摆放</t>
         </is>
       </c>
-      <c r="B1" s="169" t="n"/>
-      <c r="C1" s="169" t="n"/>
-      <c r="D1" s="169" t="n"/>
-      <c r="E1" s="169" t="n"/>
-      <c r="F1" s="169" t="n"/>
-      <c r="G1" s="169" t="n"/>
-      <c r="H1" s="169" t="n"/>
-      <c r="I1" s="169" t="n"/>
-      <c r="J1" s="169" t="n"/>
-      <c r="K1" s="169" t="n"/>
-      <c r="L1" s="179" t="n"/>
+      <c r="B1" s="170" t="n"/>
+      <c r="C1" s="170" t="n"/>
+      <c r="D1" s="170" t="n"/>
+      <c r="E1" s="170" t="n"/>
+      <c r="F1" s="170" t="n"/>
+      <c r="G1" s="170" t="n"/>
+      <c r="H1" s="170" t="n"/>
+      <c r="I1" s="170" t="n"/>
+      <c r="J1" s="170" t="n"/>
+      <c r="K1" s="170" t="n"/>
+      <c r="L1" s="180" t="n"/>
     </row>
     <row r="2" ht="14.75" customFormat="1" customHeight="1" s="1">
       <c r="A2" s="57" t="inlineStr">
@@ -6028,7 +6031,7 @@
           <t>F5505</t>
         </is>
       </c>
-      <c r="E3" s="180" t="inlineStr">
+      <c r="E3" s="181" t="inlineStr">
         <is>
           <t>三</t>
         </is>
@@ -6038,7 +6041,7 @@
           <t>F5604</t>
         </is>
       </c>
-      <c r="G3" s="180" t="inlineStr">
+      <c r="G3" s="181" t="inlineStr">
         <is>
           <t>四</t>
         </is>
@@ -6048,7 +6051,7 @@
           <t>F5608</t>
         </is>
       </c>
-      <c r="I3" s="180" t="inlineStr">
+      <c r="I3" s="181" t="inlineStr">
         <is>
           <t>五</t>
         </is>
@@ -6058,7 +6061,7 @@
           <t>F5703</t>
         </is>
       </c>
-      <c r="K3" s="181" t="inlineStr">
+      <c r="K3" s="182" t="inlineStr">
         <is>
           <t>六</t>
         </is>
@@ -6070,37 +6073,37 @@
       </c>
     </row>
     <row r="4" customFormat="1" s="1">
-      <c r="A4" s="173" t="n"/>
+      <c r="A4" s="174" t="n"/>
       <c r="B4" s="66" t="inlineStr">
         <is>
           <t>F5502</t>
         </is>
       </c>
-      <c r="C4" s="173" t="n"/>
+      <c r="C4" s="174" t="n"/>
       <c r="D4" s="67" t="inlineStr">
         <is>
           <t>F5601</t>
         </is>
       </c>
-      <c r="E4" s="173" t="n"/>
+      <c r="E4" s="174" t="n"/>
       <c r="F4" s="68" t="inlineStr">
         <is>
           <t>F5605</t>
         </is>
       </c>
-      <c r="G4" s="173" t="n"/>
+      <c r="G4" s="174" t="n"/>
       <c r="H4" s="69" t="inlineStr">
         <is>
           <t>F5609</t>
         </is>
       </c>
-      <c r="I4" s="173" t="n"/>
+      <c r="I4" s="174" t="n"/>
       <c r="J4" s="70" t="inlineStr">
         <is>
           <t>F5704</t>
         </is>
       </c>
-      <c r="K4" s="173" t="n"/>
+      <c r="K4" s="174" t="n"/>
       <c r="L4" s="72" t="inlineStr">
         <is>
           <t>F5708</t>
@@ -6108,37 +6111,37 @@
       </c>
     </row>
     <row r="5" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A5" s="173" t="n"/>
+      <c r="A5" s="174" t="n"/>
       <c r="B5" s="73" t="inlineStr">
         <is>
           <t>F5503</t>
         </is>
       </c>
-      <c r="C5" s="173" t="n"/>
+      <c r="C5" s="174" t="n"/>
       <c r="D5" s="73" t="inlineStr">
         <is>
           <t>F5602</t>
         </is>
       </c>
-      <c r="E5" s="173" t="n"/>
+      <c r="E5" s="174" t="n"/>
       <c r="F5" s="61" t="inlineStr">
         <is>
           <t>F5606</t>
         </is>
       </c>
-      <c r="G5" s="173" t="n"/>
+      <c r="G5" s="174" t="n"/>
       <c r="H5" s="74" t="inlineStr">
         <is>
           <t>F5610</t>
         </is>
       </c>
-      <c r="I5" s="173" t="n"/>
+      <c r="I5" s="174" t="n"/>
       <c r="J5" s="70" t="inlineStr">
         <is>
           <t>F5705</t>
         </is>
       </c>
-      <c r="K5" s="173" t="n"/>
+      <c r="K5" s="174" t="n"/>
       <c r="L5" s="75" t="inlineStr">
         <is>
           <t>F5709</t>
@@ -6146,37 +6149,37 @@
       </c>
     </row>
     <row r="6" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A6" s="173" t="n"/>
+      <c r="A6" s="174" t="n"/>
       <c r="B6" s="73" t="inlineStr">
         <is>
           <t>F5504</t>
         </is>
       </c>
-      <c r="C6" s="173" t="n"/>
+      <c r="C6" s="174" t="n"/>
       <c r="D6" s="73" t="inlineStr">
         <is>
           <t>F5603</t>
         </is>
       </c>
-      <c r="E6" s="173" t="n"/>
+      <c r="E6" s="174" t="n"/>
       <c r="F6" s="61" t="inlineStr">
         <is>
           <t>F5607</t>
         </is>
       </c>
-      <c r="G6" s="173" t="n"/>
+      <c r="G6" s="174" t="n"/>
       <c r="H6" s="76" t="inlineStr">
         <is>
           <t>F5701</t>
         </is>
       </c>
-      <c r="I6" s="173" t="n"/>
+      <c r="I6" s="174" t="n"/>
       <c r="J6" s="77" t="inlineStr">
         <is>
           <t>F5706</t>
         </is>
       </c>
-      <c r="K6" s="173" t="n"/>
+      <c r="K6" s="174" t="n"/>
       <c r="L6" s="78" t="inlineStr">
         <is>
           <t>F5801</t>
@@ -6184,37 +6187,37 @@
       </c>
     </row>
     <row r="7" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A7" s="173" t="n"/>
+      <c r="A7" s="174" t="n"/>
       <c r="B7" s="73" t="inlineStr">
         <is>
           <t>M5601</t>
         </is>
       </c>
-      <c r="C7" s="173" t="n"/>
+      <c r="C7" s="174" t="n"/>
       <c r="D7" s="73" t="inlineStr">
         <is>
           <t>M5705</t>
         </is>
       </c>
-      <c r="E7" s="173" t="n"/>
+      <c r="E7" s="174" t="n"/>
       <c r="F7" s="61" t="inlineStr">
         <is>
           <t>M5711</t>
         </is>
       </c>
-      <c r="G7" s="173" t="n"/>
+      <c r="G7" s="174" t="n"/>
       <c r="H7" s="79" t="inlineStr">
         <is>
           <t>F5702</t>
         </is>
       </c>
-      <c r="I7" s="173" t="n"/>
+      <c r="I7" s="174" t="n"/>
       <c r="J7" s="80" t="inlineStr">
         <is>
           <t>M5812</t>
         </is>
       </c>
-      <c r="K7" s="173" t="n"/>
+      <c r="K7" s="174" t="n"/>
       <c r="L7" s="78" t="inlineStr">
         <is>
           <t>F5802</t>
@@ -6222,37 +6225,37 @@
       </c>
     </row>
     <row r="8" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A8" s="173" t="n"/>
+      <c r="A8" s="174" t="n"/>
       <c r="B8" s="73" t="inlineStr">
         <is>
           <t>M5602</t>
         </is>
       </c>
-      <c r="C8" s="173" t="n"/>
+      <c r="C8" s="174" t="n"/>
       <c r="D8" s="73" t="inlineStr">
         <is>
           <t>M5706</t>
         </is>
       </c>
-      <c r="E8" s="173" t="n"/>
+      <c r="E8" s="174" t="n"/>
       <c r="F8" s="61" t="inlineStr">
         <is>
           <t>M5801</t>
         </is>
       </c>
-      <c r="G8" s="173" t="n"/>
+      <c r="G8" s="174" t="n"/>
       <c r="H8" s="81" t="inlineStr">
         <is>
           <t>M5806</t>
         </is>
       </c>
-      <c r="I8" s="173" t="n"/>
+      <c r="I8" s="174" t="n"/>
       <c r="J8" s="82" t="inlineStr">
         <is>
           <t>M5813</t>
         </is>
       </c>
-      <c r="K8" s="173" t="n"/>
+      <c r="K8" s="174" t="n"/>
       <c r="L8" s="78" t="inlineStr">
         <is>
           <t>F5803</t>
@@ -6260,37 +6263,37 @@
       </c>
     </row>
     <row r="9" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A9" s="173" t="n"/>
+      <c r="A9" s="174" t="n"/>
       <c r="B9" s="73" t="inlineStr">
         <is>
           <t>M5701</t>
         </is>
       </c>
-      <c r="C9" s="173" t="n"/>
+      <c r="C9" s="174" t="n"/>
       <c r="D9" s="73" t="inlineStr">
         <is>
           <t>M5707</t>
         </is>
       </c>
-      <c r="E9" s="173" t="n"/>
+      <c r="E9" s="174" t="n"/>
       <c r="F9" s="61" t="inlineStr">
         <is>
           <t>M5802</t>
         </is>
       </c>
-      <c r="G9" s="173" t="n"/>
+      <c r="G9" s="174" t="n"/>
       <c r="H9" s="83" t="inlineStr">
         <is>
           <t>M5807</t>
         </is>
       </c>
-      <c r="I9" s="173" t="n"/>
+      <c r="I9" s="174" t="n"/>
       <c r="J9" s="84" t="inlineStr">
         <is>
           <t>M5814</t>
         </is>
       </c>
-      <c r="K9" s="173" t="n"/>
+      <c r="K9" s="174" t="n"/>
       <c r="L9" s="78" t="inlineStr">
         <is>
           <t>M5903</t>
@@ -6299,37 +6302,37 @@
       <c r="O9" s="85" t="n"/>
     </row>
     <row r="10" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A10" s="173" t="n"/>
+      <c r="A10" s="174" t="n"/>
       <c r="B10" s="73" t="inlineStr">
         <is>
           <t>M5702</t>
         </is>
       </c>
-      <c r="C10" s="173" t="n"/>
+      <c r="C10" s="174" t="n"/>
       <c r="D10" s="86" t="inlineStr">
         <is>
           <t>M5708</t>
         </is>
       </c>
-      <c r="E10" s="173" t="n"/>
+      <c r="E10" s="174" t="n"/>
       <c r="F10" s="61" t="inlineStr">
         <is>
           <t>M5803</t>
         </is>
       </c>
-      <c r="G10" s="173" t="n"/>
+      <c r="G10" s="174" t="n"/>
       <c r="H10" s="70" t="inlineStr">
         <is>
           <t>M5808</t>
         </is>
       </c>
-      <c r="I10" s="173" t="n"/>
+      <c r="I10" s="174" t="n"/>
       <c r="J10" s="87" t="inlineStr">
         <is>
           <t>M5815</t>
         </is>
       </c>
-      <c r="K10" s="173" t="n"/>
+      <c r="K10" s="174" t="n"/>
       <c r="L10" s="78" t="inlineStr">
         <is>
           <t>M5904</t>
@@ -6337,37 +6340,37 @@
       </c>
     </row>
     <row r="11" customFormat="1" s="1">
-      <c r="A11" s="173" t="n"/>
+      <c r="A11" s="174" t="n"/>
       <c r="B11" s="73" t="inlineStr">
         <is>
           <t>M5703</t>
         </is>
       </c>
-      <c r="C11" s="173" t="n"/>
+      <c r="C11" s="174" t="n"/>
       <c r="D11" s="86" t="inlineStr">
         <is>
           <t>M5709</t>
         </is>
       </c>
-      <c r="E11" s="173" t="n"/>
+      <c r="E11" s="174" t="n"/>
       <c r="F11" s="61" t="inlineStr">
         <is>
           <t>M5804</t>
         </is>
       </c>
-      <c r="G11" s="173" t="n"/>
+      <c r="G11" s="174" t="n"/>
       <c r="H11" s="88" t="inlineStr">
         <is>
           <t>M5809</t>
         </is>
       </c>
-      <c r="I11" s="173" t="n"/>
+      <c r="I11" s="174" t="n"/>
       <c r="J11" s="89" t="inlineStr">
         <is>
           <t>M5901</t>
         </is>
       </c>
-      <c r="K11" s="173" t="n"/>
+      <c r="K11" s="174" t="n"/>
       <c r="L11" s="90" t="inlineStr">
         <is>
           <t>M5905</t>
@@ -6375,37 +6378,37 @@
       </c>
     </row>
     <row r="12" customFormat="1" s="1">
-      <c r="A12" s="173" t="n"/>
+      <c r="A12" s="174" t="n"/>
       <c r="B12" s="73" t="inlineStr">
         <is>
           <t>M5704</t>
         </is>
       </c>
-      <c r="C12" s="173" t="n"/>
+      <c r="C12" s="174" t="n"/>
       <c r="D12" s="73" t="inlineStr">
         <is>
           <t>M5710</t>
         </is>
       </c>
-      <c r="E12" s="173" t="n"/>
+      <c r="E12" s="174" t="n"/>
       <c r="F12" s="61" t="inlineStr">
         <is>
           <t>M5805</t>
         </is>
       </c>
-      <c r="G12" s="173" t="n"/>
+      <c r="G12" s="174" t="n"/>
       <c r="H12" s="91" t="inlineStr">
         <is>
           <t>M5810</t>
         </is>
       </c>
-      <c r="I12" s="173" t="n"/>
+      <c r="I12" s="174" t="n"/>
       <c r="J12" s="60" t="inlineStr">
         <is>
           <t>M5902</t>
         </is>
       </c>
-      <c r="K12" s="173" t="n"/>
+      <c r="K12" s="174" t="n"/>
       <c r="L12" s="92" t="inlineStr">
         <is>
           <t>M6001</t>
@@ -6413,21 +6416,21 @@
       </c>
     </row>
     <row r="13" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A13" s="176" t="n"/>
+      <c r="A13" s="177" t="n"/>
       <c r="B13" s="93" t="n"/>
-      <c r="C13" s="176" t="n"/>
+      <c r="C13" s="177" t="n"/>
       <c r="D13" s="93" t="n"/>
-      <c r="E13" s="176" t="n"/>
+      <c r="E13" s="177" t="n"/>
       <c r="F13" s="93" t="n"/>
-      <c r="G13" s="176" t="n"/>
+      <c r="G13" s="177" t="n"/>
       <c r="H13" s="94" t="inlineStr">
         <is>
           <t>M5811</t>
         </is>
       </c>
-      <c r="I13" s="176" t="n"/>
+      <c r="I13" s="177" t="n"/>
       <c r="J13" s="94" t="n"/>
-      <c r="K13" s="176" t="n"/>
+      <c r="K13" s="177" t="n"/>
       <c r="L13" s="94" t="inlineStr">
         <is>
           <t>M6002</t>
@@ -6482,24 +6485,24 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A1" s="182" t="inlineStr">
+      <c r="A1" s="183" t="inlineStr">
         <is>
           <t>马靴摆放</t>
         </is>
       </c>
-      <c r="B1" s="183" t="n"/>
-      <c r="C1" s="183" t="n"/>
-      <c r="D1" s="183" t="n"/>
-      <c r="E1" s="183" t="n"/>
-      <c r="F1" s="183" t="n"/>
-      <c r="G1" s="183" t="n"/>
-      <c r="H1" s="183" t="n"/>
-      <c r="I1" s="183" t="n"/>
-      <c r="J1" s="183" t="n"/>
-      <c r="K1" s="183" t="n"/>
-      <c r="L1" s="183" t="n"/>
-      <c r="M1" s="183" t="n"/>
-      <c r="N1" s="184" t="n"/>
+      <c r="B1" s="184" t="n"/>
+      <c r="C1" s="184" t="n"/>
+      <c r="D1" s="184" t="n"/>
+      <c r="E1" s="184" t="n"/>
+      <c r="F1" s="184" t="n"/>
+      <c r="G1" s="184" t="n"/>
+      <c r="H1" s="184" t="n"/>
+      <c r="I1" s="184" t="n"/>
+      <c r="J1" s="184" t="n"/>
+      <c r="K1" s="184" t="n"/>
+      <c r="L1" s="184" t="n"/>
+      <c r="M1" s="184" t="n"/>
+      <c r="N1" s="185" t="n"/>
     </row>
     <row r="2" customFormat="1" s="1">
       <c r="A2" s="5" t="inlineStr">
@@ -6651,7 +6654,7 @@
           <t>置物架</t>
         </is>
       </c>
-      <c r="C4" s="185" t="n"/>
+      <c r="C4" s="186" t="n"/>
       <c r="D4" s="23" t="inlineStr">
         <is>
           <t>X43-03</t>
@@ -6692,16 +6695,16 @@
           <t>N42/43.5-01</t>
         </is>
       </c>
-      <c r="L4" s="186" t="inlineStr">
+      <c r="L4" s="187" t="inlineStr">
         <is>
           <t>置物架</t>
         </is>
       </c>
-      <c r="N4" s="185" t="n"/>
+      <c r="N4" s="186" t="n"/>
     </row>
     <row r="5" customFormat="1" s="1">
-      <c r="A5" s="187" t="n"/>
-      <c r="C5" s="185" t="n"/>
+      <c r="A5" s="188" t="n"/>
+      <c r="C5" s="186" t="n"/>
       <c r="D5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">X43-02 </t>
@@ -6742,12 +6745,12 @@
           <t>N42/42.5-01 张子恒</t>
         </is>
       </c>
-      <c r="L5" s="188" t="n"/>
-      <c r="N5" s="185" t="n"/>
+      <c r="L5" s="189" t="n"/>
+      <c r="N5" s="186" t="n"/>
     </row>
     <row r="6" customFormat="1" s="1">
-      <c r="A6" s="187" t="n"/>
-      <c r="C6" s="185" t="n"/>
+      <c r="A6" s="188" t="n"/>
+      <c r="C6" s="186" t="n"/>
       <c r="D6" s="27" t="inlineStr">
         <is>
           <t>X43-01</t>
@@ -6788,13 +6791,13 @@
           <t xml:space="preserve">N42/40.5-01 </t>
         </is>
       </c>
-      <c r="L6" s="188" t="n"/>
-      <c r="N6" s="185" t="n"/>
+      <c r="L6" s="189" t="n"/>
+      <c r="N6" s="186" t="n"/>
     </row>
     <row r="7" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A7" s="189" t="n"/>
-      <c r="B7" s="190" t="n"/>
-      <c r="C7" s="191" t="n"/>
+      <c r="A7" s="190" t="n"/>
+      <c r="B7" s="191" t="n"/>
+      <c r="C7" s="192" t="n"/>
       <c r="D7" s="18" t="inlineStr">
         <is>
           <t>X42-24</t>
@@ -6835,9 +6838,9 @@
           <t>N41/42-01 （舟山）</t>
         </is>
       </c>
-      <c r="L7" s="192" t="n"/>
-      <c r="M7" s="190" t="n"/>
-      <c r="N7" s="191" t="n"/>
+      <c r="L7" s="193" t="n"/>
+      <c r="M7" s="191" t="n"/>
+      <c r="N7" s="192" t="n"/>
     </row>
     <row r="8" ht="14.75" customFormat="1" customHeight="1" s="1">
       <c r="A8" s="30" t="n"/>
@@ -6885,7 +6888,7 @@
           <t>置物架</t>
         </is>
       </c>
-      <c r="B9" s="184" t="n"/>
+      <c r="B9" s="185" t="n"/>
       <c r="C9" s="39" t="n"/>
       <c r="D9" s="40" t="n"/>
       <c r="E9" s="38" t="inlineStr">
@@ -6940,8 +6943,8 @@
       </c>
     </row>
     <row r="10" customFormat="1" s="1">
-      <c r="A10" s="187" t="n"/>
-      <c r="B10" s="185" t="n"/>
+      <c r="A10" s="188" t="n"/>
+      <c r="B10" s="186" t="n"/>
       <c r="C10" s="45" t="n"/>
       <c r="D10" s="8" t="inlineStr">
         <is>
@@ -7000,8 +7003,8 @@
       </c>
     </row>
     <row r="11" customFormat="1" s="1">
-      <c r="A11" s="187" t="n"/>
-      <c r="B11" s="185" t="n"/>
+      <c r="A11" s="188" t="n"/>
+      <c r="B11" s="186" t="n"/>
       <c r="C11" s="47" t="inlineStr">
         <is>
           <t>X45-01</t>
@@ -7064,8 +7067,8 @@
       </c>
     </row>
     <row r="12" ht="14.75" customFormat="1" customHeight="1" s="1">
-      <c r="A12" s="189" t="n"/>
-      <c r="B12" s="191" t="n"/>
+      <c r="A12" s="190" t="n"/>
+      <c r="B12" s="192" t="n"/>
       <c r="C12" s="22" t="inlineStr">
         <is>
           <t>X39-03 张鹏</t>

</xml_diff>